<commit_message>
Add Fixture Master Plan UI and fix Control Plan image handling
</commit_message>
<xml_diff>
--- a/metalman-auto-engineer/backend/outputs/Tooling_List_92187158.xlsx
+++ b/metalman-auto-engineer/backend/outputs/Tooling_List_92187158.xlsx
@@ -725,6 +725,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -750,6 +753,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -775,6 +781,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -800,6 +809,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1099,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22.36328125" customWidth="1" style="2" min="1" max="1"/>
@@ -1340,7 +1352,7 @@
       </c>
       <c r="L8" s="39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>100</t>
         </is>
       </c>
       <c r="M8" s="48" t="n"/>
@@ -1499,8 +1511,6 @@
     <row r="12" ht="327" customFormat="1" customHeight="1" s="2">
       <c r="C12" s="1" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14"/>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="L8:N8"/>

</xml_diff>